<commit_message>
style: remove green highlight on Live status cells across master workbooks and provide 1-click Apps Script removal
</commit_message>
<xml_diff>
--- a/05_STREAMING_PORTAL/Google_Sheets_Complete_Master.xlsx
+++ b/05_STREAMING_PORTAL/Google_Sheets_Complete_Master.xlsx
@@ -34,8 +34,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="0015803D"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -44,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -55,12 +54,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="001E293B"/>
         <bgColor rgb="001E293B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -87,10 +80,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
feat: in-browser web app stream audit, keep only web-app playable streams in Sheet 1, move dead/unplayable to Sheet 2, and remove VLC/mobile prompts
</commit_message>
<xml_diff>
--- a/05_STREAMING_PORTAL/Google_Sheets_Complete_Master.xlsx
+++ b/05_STREAMING_PORTAL/Google_Sheets_Complete_Master.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -525,19 +525,19 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Fail Army</t>
+          <t>Isaiaruvi Tv</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://failarmy-international-in.samsung.wurl.tv/playlist.m3u8</t>
+          <t>https://segment.yuppcdn.net/140622/isaiaruvi/playlist.m3u8</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -552,46 +552,46 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hungama TV</t>
+          <t>Kalaignar Tv</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>http://103.185.24.134:3001/HUNGAMA/index.m3u8</t>
+          <t>https://segment.yuppcdn.net/240122/kalaignartv/playlist.m3u8</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>👶</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Isaiaruvi Tv</t>
+          <t>Life TV</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/140622/isaiaruvi/playlist.m3u8</t>
+          <t>https://lifetv.livebox.co.in/lifetvhls/lifetv.m3u8</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -606,19 +606,19 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Kalaignar Tv</t>
+          <t>Mei Alai TV</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/240122/kalaignartv/playlist.m3u8</t>
+          <t>https://meialai.iptelevishion.com/meialai/2/index.m3u8</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -633,46 +633,46 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Life TV</t>
+          <t>Movie Club Tv</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://lifetv.livebox.co.in/lifetvhls/lifetv.m3u8</t>
+          <t>https://sis-global.prod.samsungtv.plus/v1/tvpprd/sc-mp2ar4ca425xo.m3u8</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Mei Alai TV</t>
+          <t>Murasu Tv</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://meialai.iptelevishion.com/meialai/2/index.m3u8</t>
+          <t>https://segment.yuppcdn.net/050522/murasu/playlist.m3u8</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -687,46 +687,46 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Movie Club 2 Tv</t>
+          <t>NH Tamil Gold</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://d3gnyty2vddhsg.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-ytipwjqub3kf8/TMC2_IN.m3u8?ads.ads_cdn=cf&amp;ads.cdn=cf</t>
+          <t>https://d3arbp6l7f096k.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-gv6wgpbb4mgwk/playlist.m3u8?ads.ads_cdn=cf&amp;ads.app_domain=APP_DOMAIN&amp;ads.cdn=cf</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Movie Club Tv</t>
+          <t>OM TV</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://sis-global.prod.samsungtv.plus/v1/tvpprd/sc-mp2ar4ca425xo.m3u8</t>
+          <t>https://mumt01.tangotv.in/O5aw8Zn3OMTV/index.m3u8</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -741,19 +741,19 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Murasu Tv</t>
+          <t>Puthuyugam TV</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://segment.yuppcdn.net/050522/murasu/playlist.m3u8</t>
+          <t>https://mumt04.tangotv.in/m18aqlK4PUTHUYUGAMTV/index.m3u8</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -768,19 +768,19 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>NH Tamil Gold</t>
+          <t>Roja TV2</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://d3arbp6l7f096k.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-gv6wgpbb4mgwk/playlist.m3u8?ads.ads_cdn=cf&amp;ads.app_domain=APP_DOMAIN&amp;ads.cdn=cf</t>
+          <t>https://stream.rojatv.cloud/rojatv/rojatv/index.m3u8</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -795,19 +795,19 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Nickelodeon</t>
+          <t>Sirippoli TV2</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>http://103.185.24.134:3001/NICK/index.m3u8</t>
+          <t>https://yuppmedtaorire.akamaized.net/v1/manifest/a0d007312bfd99c47f76b77ae26b1ccdaae76cb1/siripoli_nim_https/c4e6500f-ea05-4226-810e-2833ee0075ff/0.m3u8</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -822,73 +822,73 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>OM TV</t>
+          <t>Sivan TV</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://mumt01.tangotv.in/O5aw8Zn3OMTV/index.m3u8</t>
+          <t>https://sivantv.livebox.co.in/sivantvhls/sivan.m3u8</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Polimer TV</t>
+          <t>South Station Tv</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1241/master.m3u8</t>
+          <t>https://cc-yw7ztecy8do3q.akamaized.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/cc-yw7ztecy8do3q/SS_IN.m3u8</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Puthuyugam TV</t>
+          <t>Thalaa Tv</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://mumt04.tangotv.in/m18aqlK4PUTHUYUGAMTV/index.m3u8</t>
+          <t>https://streams2.sofast.tv/ptnr-yupptv/title-THALAA-TV-TAM/sofastplayout/981f8f06-782a-4962-b5e0-7dcccd65279c_0_HLS/manifest.m3u8</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -903,19 +903,19 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Roja TV2</t>
+          <t>Ultimate TV2</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://stream.rojatv.cloud/rojatv/rojatv/index.m3u8</t>
+          <t>https://mumbai-edge.smartplaytv.in/utv/index.m3u8</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -930,19 +930,19 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Sai TV</t>
+          <t>Vaanavil Tv</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://mumt03.tangotv.in/Dsly5z3HSAITV/index.m3u8</t>
+          <t>https://6n3yope4d9ok-hls-live.5centscdn.com/vaanavil/TV.stream/playlist.m3u8</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -957,19 +957,19 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Sirippoli TV2</t>
+          <t>WOW Kidz Tamil</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://yuppmedtaorire.akamaized.net/v1/manifest/a0d007312bfd99c47f76b77ae26b1ccdaae76cb1/siripoli_nim_https/c4e6500f-ea05-4226-810e-2833ee0075ff/0.m3u8</t>
+          <t>https://yuppparoriglin.akamaized.net/181224/smil:wowkidztam.smil/playlist.m3u8?hdnts=st=1735898689~exp=1835898688~acl=*~hmac=f5fe24724fe05481e3841f9eb5ab8efdee0a3dd83645ae9dcf45703f525bab7b</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -984,73 +984,73 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Sivan TV</t>
+          <t>Zee South Flix Tv</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>https://sivantv.livebox.co.in/sivantvhls/sivan.m3u8</t>
+          <t>https://amg00862-amg00862c9-amgplt0173.playout.now3.amagi.tv/playlist/amg00862-amg00862c9-amgplt0173/playlist.m3u8</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Sony Sports Ten 4</t>
+          <t>Zee Tamil HD</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://cloudplay-sonyliv.pages.dev/ten4.m3u8</t>
+          <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:zeetamil1.smil/playlist.m3u8</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>South Station Tv</t>
+          <t>MK Six TV2</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://cc-yw7ztecy8do3q.akamaized.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/cc-yw7ztecy8do3q/SS_IN.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1253/master.m3u8</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1065,154 +1065,154 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Super Hungama</t>
+          <t>Peppers Tv</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>http://103.185.24.134:3001/SUPER-HUNGAMA/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1383/master.m3u8</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>👶</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Thalaa Tv</t>
+          <t>Puthiyathalaimurai tv</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://streams2.sofast.tv/ptnr-yupptv/title-THALAA-TV-TAM/sofastplayout/981f8f06-782a-4962-b5e0-7dcccd65279c_0_HLS/manifest.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1261/master.m3u8</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Toonami Movie</t>
+          <t>Raj Musix Tamil</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>http://api.toonamiaftermath.com:3000/movies/playlist.m3u8</t>
+          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/Raj_Musix/master_1.m3u8</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>👶</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Ultimate TV2</t>
+          <t>Shemaroo Tv</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>https://mumbai-edge.smartplaytv.in/utv/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/230/master.m3u8</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Vaanavil Tv</t>
+          <t>Studio One Tv</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>https://6n3yope4d9ok-hls-live.5centscdn.com/vaanavil/TV.stream/playlist.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/276/master.m3u8</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>WOW Kidz Tamil</t>
+          <t>Suriya Tv</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://yuppparoriglin.akamaized.net/181224/smil:wowkidztam.smil/playlist.m3u8?hdnts=st=1735898689~exp=1835898688~acl=*~hmac=f5fe24724fe05481e3841f9eb5ab8efdee0a3dd83645ae9dcf45703f525bab7b</t>
+          <t>https://stream.ottlive.co.in/suryatvtamil/index.m3u8</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1227,100 +1227,100 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Zee South Flix Tv</t>
+          <t>Thanthi Tv</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>https://amg00862-amg00862c9-amgplt0173.playout.now3.amagi.tv/playlist/amg00862-amg00862c9-amgplt0173/playlist.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1612/master.m3u8</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Zee Tamil HD</t>
+          <t>Velicham Tv</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>https://da86m1sqpm3o0.cloudfront.net/28072023/smil:zeetamil1.smil/playlist.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/461/master.m3u8</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MK Six TV2</t>
+          <t>Vendar Tv</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1253/master.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1271/master.m3u8</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>News J</t>
+          <t>DD Tamil</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1279/master.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/26/master.m3u8</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1330,24 +1330,24 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>NTC TV</t>
+          <t>Malai Murasu Tv</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>https://galaxyott.live/hls/ntv.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1606/master.m3u8</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1357,24 +1357,24 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Oli TV</t>
+          <t>Polimer news</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>https://live.olidigital.in/olitv/olitv/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1245/master.m3u8</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1384,213 +1384,213 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Peppers Tv</t>
+          <t>Rakuten Action Movies</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1383/master.m3u8</t>
+          <t>https://54045f0c40fd442c8b06df076aaf1e85.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6065/master.m3u8</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Puthiyathalaimurai tv</t>
+          <t>Rakuten Family Movies</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1261/master.m3u8</t>
+          <t>https://e3207568b726401995c25670faaf32e4.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6203/master.m3u8</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Raj Musix Tamil</t>
+          <t>Rakuten Top Movies</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/Raj_Musix/master_1.m3u8</t>
+          <t>https://0145451975a64b35866170fd2e8fa486.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-5987/master.m3u8</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Raj TV</t>
+          <t>YET TV</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/RAJTV/master_1.m3u8</t>
+          <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv.m3u8</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Shemaroo Tv</t>
+          <t>MK Six TV1</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/230/master.m3u8</t>
+          <t>https://mumt06.tangotv.in/qYyB8fXVMKSIX/index.m3u8</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Sony MAX HD</t>
+          <t>Manorama Tv</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%20HD.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1479/master.m3u8</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Studio One Tv</t>
+          <t>News 7 Tv</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/276/master.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1498/master.m3u8</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Suriya Tv</t>
+          <t>We Tv</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>https://stream.ottlive.co.in/suryatvtamil/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1530/master.m3u8</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1605,115 +1605,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Thanthi Tv</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1612/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Travel XP HD Tv</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>https://deltatesttatasky.akamaized.net/out/i/968284.m3u8</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>🌐</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Velicham Tv</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/461/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Tamil</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>📺</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Vendar Tv</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>https://cdn.pishow.tv/ott/live/1271/master.m3u8</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Malayalam</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>🪷</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1768,255 +1660,255 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Angel TV</t>
+          <t>Fail Army</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-394914/india/ngrp:angelindia_all/playlist.m3u8</t>
+          <t>https://failarmy-international-in.samsung.wurl.tv/playlist.m3u8</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>🪷</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Angel TV America</t>
+          <t>Hungama TV</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-374850/america/ngrp:angelamerica_all/playlist.m3u8</t>
+          <t>http://103.185.24.134:3001/HUNGAMA/index.m3u8</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>🪷</t>
+          <t>👶</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Angel TV Indonesia</t>
+          <t>Movie Club 2 Tv</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://janya-digimix.akamaized.net/vglive-sk-234616/indonesia/ngrp:angelindonesia_all/playlist.m3u8</t>
+          <t>https://d3gnyty2vddhsg.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/pb-ytipwjqub3kf8/TMC2_IN.m3u8?ads.ads_cdn=cf&amp;ads.cdn=cf</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>🪷</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Chithiram Tv</t>
+          <t>Nickelodeon</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1243/master.m3u8</t>
+          <t>http://103.185.24.134:3001/NICK/index.m3u8</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>👶</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DD Tamil</t>
+          <t>Polimer TV</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/26/master.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1241/master.m3u8</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DD Tamil</t>
+          <t>Sai TV</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://d2lk5u59tns74c.cloudfront.net/out/v1/abf46b148419409d8469d7a9b0c26563/index.m3u8</t>
+          <t>https://mumt03.tangotv.in/Dsly5z3HSAITV/index.m3u8</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Go USA</t>
+          <t>Sony Sports Ten 4</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://brandusa-gousa-1-in.samsung.wurl.tv/playlist.m3u8</t>
+          <t>https://cloudplay-sonyliv.pages.dev/ten4.m3u8</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Malai Murasu Tv</t>
+          <t>Super Hungama</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1606/master.m3u8</t>
+          <t>http://103.185.24.134:3001/SUPER-HUNGAMA/index.m3u8</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>👶</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Malar Tv</t>
+          <t>Toonami Movie</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/473/master.m3u8</t>
+          <t>http://api.toonamiaftermath.com:3000/movies/playlist.m3u8</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>👶</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Moon Tv</t>
+          <t>News J</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://player.mslivestream.net/mslive/e10bb900976df9177b9a080314f26f86.sdp/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1279/master.m3u8</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2026,24 +1918,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MTA6 Asia</t>
+          <t>NTC TV</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mta6asia/playlist.m3u8</t>
+          <t>https://galaxyott.live/hls/ntv.m3u8</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2053,24 +1945,24 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>🪷</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MTA7 Asia</t>
+          <t>Oli TV</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mtaasia2/playlist.m3u8</t>
+          <t>https://live.olidigital.in/olitv/olitv/index.m3u8</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2080,78 +1972,78 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>🪷</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Polimer news</t>
+          <t>Raj TV</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1245/master.m3u8</t>
+          <t>https://livestream.rajtv.tv/hlslive/Admin/px08241087/live/RAJTV/master_1.m3u8</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Polimer news</t>
+          <t>Sony MAX HD</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://live-cf-polimernews.dailyhunt.in/master.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%20HD.m3u8</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Action Movies</t>
+          <t>Travel XP HD Tv</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://54045f0c40fd442c8b06df076aaf1e85.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6065/master.m3u8</t>
+          <t>https://deltatesttatasky.akamaized.net/out/i/968284.m3u8</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2161,267 +2053,267 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🌐</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Family Movies</t>
+          <t>Chithiram Tv</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://e3207568b726401995c25670faaf32e4.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-6203/master.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1243/master.m3u8</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>👶</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Top Movies</t>
+          <t>DD Tamil</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://0145451975a64b35866170fd2e8fa486.mediatailor.eu-west-1.amazonaws.com/v1/master/0547f18649bd788bec7b67b746e47670f558b6b2/production-LiveChannel-5987/master.m3u8</t>
+          <t>https://d2lk5u59tns74c.cloudfront.net/out/v1/abf46b148419409d8469d7a9b0c26563/index.m3u8</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Sony MAX 2</t>
+          <t>Malar Tv</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%202.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/473/master.m3u8</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Sony PIX HD</t>
+          <t>Moon Tv</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20PIX%20HD.m3u8</t>
+          <t>https://player.mslivestream.net/mslive/e10bb900976df9177b9a080314f26f86.sdp/index.m3u8</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Sony WAH</t>
+          <t>Polimer news</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20WAH.m3u8</t>
+          <t>https://live-cf-polimernews.dailyhunt.in/master.m3u8</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Win Tv</t>
+          <t>Sony MAX 2</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1531/master.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20MAX%202.m3u8</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>YET TV</t>
+          <t>Sony PIX HD</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://live.yettelevision.com:5443/LiveApp/streams/yettv.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20PIX%20HD.m3u8</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>English</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Zee Tamil News</t>
+          <t>Sony WAH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/amazeyourself/adaptive-streams/refs/heads/main/streams/in/ZMCL/ZeeTamilNews.m3u8</t>
+          <t>https://sl.vodep39240327.workers.dev/channel/SONY%20WAH.m3u8</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MK Six TV1</t>
+          <t>Win Tv</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://mumt06.tangotv.in/qYyB8fXVMKSIX/index.m3u8</t>
+          <t>https://cdn.pishow.tv/ott/live/1531/master.m3u8</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>IBC Tamil</t>
+          <t>Zee Tamil News</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>https://ibc.massstream.net/IBC/index.m3u8</t>
+          <t>https://raw.githubusercontent.com/amazeyourself/adaptive-streams/refs/heads/main/streams/in/ZMCL/ZeeTamilNews.m3u8</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2431,39 +2323,39 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>📺</t>
+          <t>📰</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Manorama Tv</t>
+          <t>IBC Tamil</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1479/master.m3u8</t>
+          <t>https://ibc.massstream.net/IBC/index.m3u8</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>📺</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
@@ -2490,46 +2382,46 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>News 7 Tv</t>
+          <t>Sooriyan TV</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1498/master.m3u8</t>
+          <t>https://live20.bozztv.com/giatv/giatv-Infinittyott/Infinittyott/playlist.m3u8</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>📰</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Sooriyan TV</t>
+          <t>Star Vijay HD</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>https://live20.bozztv.com/giatv/giatv-Infinittyott/Infinittyott/playlist.m3u8</t>
+          <t>https://peaky.techcoder40.workers.dev/776.m3u8</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2544,73 +2436,73 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Star Vijay HD</t>
+          <t>Suriyan Tv</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>https://peaky.techcoder40.workers.dev/776.m3u8</t>
+          <t>https://stream.sscloud7.com/live/suriyantv/index.m3u8</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🎬</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Suriyan Tv</t>
+          <t>Vijay Takkar APAC</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>https://stream.sscloud7.com/live/suriyantv/index.m3u8</t>
+          <t>https://tglmp01.akamaized.net/out/v1/c1071012b73f4f189b202e1529e8f802/manifest.mpd</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>🎬</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Vijay Takkar APAC</t>
+          <t>Angel TV</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>https://tglmp01.akamaized.net/out/v1/c1071012b73f4f189b202e1529e8f802/manifest.mpd</t>
+          <t>https://janya-digimix.akamaized.net/vglive-sk-394914/india/ngrp:angelindia_all/playlist.m3u8</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2620,39 +2512,147 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>We Tv</t>
+          <t>Angel TV America</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>https://cdn.pishow.tv/ott/live/1530/master.m3u8</t>
+          <t>https://janya-digimix.akamaized.net/vglive-sk-374850/america/ngrp:angelamerica_all/playlist.m3u8</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>🎵</t>
+          <t>🪷</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Dead</t>
+          <t>DEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Angel TV Indonesia</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>https://janya-digimix.akamaized.net/vglive-sk-234616/indonesia/ngrp:angelindonesia_all/playlist.m3u8</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>🪷</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Go USA</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>https://brandusa-gousa-1-in.samsung.wurl.tv/playlist.m3u8</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>🎬</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>MTA6 Asia</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mta6asia/playlist.m3u8</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>🪷</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>MTA7 Asia</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>https://livemtaasia.akamaized.net/hls/live/2039224/mtaasia2/playlist.m3u8</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>🪷</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>DEAD</t>
         </is>
       </c>
     </row>

</xml_diff>